<commit_message>
Add Polo colours and correct oversized sizing
</commit_message>
<xml_diff>
--- a/Products/TShirts/The Numbered/Oversized/Size Chart.xlsx
+++ b/Products/TShirts/The Numbered/Oversized/Size Chart.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\Denied\Products\Oversized\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\Denied\Products\TShirts\The Numbered\Oversized\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B034A25-80EB-411A-A46A-1814BAD59FBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CC8144C-D77A-4C6F-8D0C-D426A1748A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32856" yWindow="912" windowWidth="34560" windowHeight="18600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Size</t>
   </si>
@@ -52,9 +52,6 @@
   </si>
   <si>
     <t>XS</t>
-  </si>
-  <si>
-    <t>XXXL</t>
   </si>
 </sst>
 </file>
@@ -416,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -438,7 +435,7 @@
         <v>39</v>
       </c>
       <c r="C2" s="1">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -449,7 +446,7 @@
         <v>41</v>
       </c>
       <c r="C3" s="1">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -460,7 +457,7 @@
         <v>43</v>
       </c>
       <c r="C4" s="1">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -471,7 +468,7 @@
         <v>45</v>
       </c>
       <c r="C5" s="1">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -482,7 +479,7 @@
         <v>47</v>
       </c>
       <c r="C6" s="1">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -493,17 +490,6 @@
         <v>49</v>
       </c>
       <c r="C7" s="1">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="1">
-        <v>51</v>
-      </c>
-      <c r="C8" s="1">
         <v>32</v>
       </c>
     </row>

</xml_diff>